<commit_message>
[Add item rips json]
</commit_message>
<xml_diff>
--- a/descarga_documentos_magaly/RipsInfoFebrero.xlsx
+++ b/descarga_documentos_magaly/RipsInfoFebrero.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\script_node\descarga_documentos_magaly\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EF95885-FBBD-4470-9284-AD9EF9E57AF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D756E193-6207-46DD-AB19-AAC43BFE6DB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="225">
   <si>
     <t>numFactura</t>
   </si>
@@ -597,6 +597,117 @@
   </si>
   <si>
     <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/rta_api_cuv_9506014d8f0cd8f97b77a60f85cd38323e4fb5cd3bffe05ed46cbc4d586e18e29daf6e0739c20e2f09edcfc6ea3feb21.json</t>
+  </si>
+  <si>
+    <t>valor_total_reteiva</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy21629359769a9e382a85f8.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy59046586169a9e38d02ad5.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/06/contenido_json_rips_OTAwODEwNDAy194946262869aaeaffc8344.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy99191036369a9e3731903c.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy130340609869a9e42e3f690.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy172596743969a9e392ad46f.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy163521214569a9e433e67fc.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy193069166569a9e37d71bdc.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy130546381569a9e41db4713.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy76035945469a9e3ab714ca.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy22375480469a9e387b7a9b.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy77194354469a9e36da4adf.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy19484554069a9e44480fe6.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy139680948769a9e39ea547b.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy185375257369a9e44a22985.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy101755341369a9e3685cb96.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy122580558869a9e428a7731.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy28993833369a9e39886eaf.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy66678647469a9e43ed16af.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy156736247769a9e362c7982.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/06/contenido_json_rips_OTAwODEwNDAy63594907669aaeaf6d8f26.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy44812750769a9e40d017d6.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy198067800069a9e412c00d4.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy204365738169a9e5421babf.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy58446541369a9e43924112.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy117774575769a9e47cd3d76.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy165052997669a9e45acd6a0.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy38210805869a9e42305d71.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy205502910369a9e4603a051.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy52822377269a9e4552dbe0.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy16788635969a9e4fde6d45.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy144694104869a9e4046a640.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy22782394169a9e4184e719.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/06/contenido_json_rips_OTAwODEwNDAy134014083469aaeafd30468.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy1087786869a9e37840761.json</t>
+  </si>
+  <si>
+    <t>https://afacturar.archivamos.com/d31e58d5/b2506588230995c21583bdd64afbdef147112036/rips/2026/03/05/contenido_json_rips_OTAwODEwNDAy188538538369a9e44f8450d.json</t>
   </si>
 </sst>
 </file>
@@ -1464,14 +1575,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="4" max="4" width="82.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="85.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.08984375" customWidth="1"/>
+    <col min="5" max="5" width="27.7265625" customWidth="1"/>
+    <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.7265625" customWidth="1"/>
+    <col min="8" max="8" width="151.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1493,8 +1607,11 @@
       <c r="G1" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H1" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1516,8 +1633,11 @@
       <c r="G2" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -1539,8 +1659,11 @@
       <c r="G3" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H3" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -1562,8 +1685,11 @@
       <c r="G4" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H4" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -1585,8 +1711,11 @@
       <c r="G5" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H5" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -1608,8 +1737,11 @@
       <c r="G6" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H6" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>23</v>
       </c>
@@ -1631,8 +1763,11 @@
       <c r="G7" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H7" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>27</v>
       </c>
@@ -1654,8 +1789,11 @@
       <c r="G8" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H8" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>31</v>
       </c>
@@ -1677,8 +1815,11 @@
       <c r="G9" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H9" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>35</v>
       </c>
@@ -1700,8 +1841,11 @@
       <c r="G10" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H10" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>39</v>
       </c>
@@ -1723,8 +1867,11 @@
       <c r="G11" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H11" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>43</v>
       </c>
@@ -1746,8 +1893,11 @@
       <c r="G12" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H12" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>47</v>
       </c>
@@ -1769,8 +1919,11 @@
       <c r="G13" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H13" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>51</v>
       </c>
@@ -1792,8 +1945,11 @@
       <c r="G14" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H14" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>55</v>
       </c>
@@ -1815,8 +1971,11 @@
       <c r="G15" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H15" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>59</v>
       </c>
@@ -1838,8 +1997,11 @@
       <c r="G16" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H16" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>63</v>
       </c>
@@ -1861,8 +2023,11 @@
       <c r="G17" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H17" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>67</v>
       </c>
@@ -1884,8 +2049,11 @@
       <c r="G18" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H18" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>71</v>
       </c>
@@ -1907,8 +2075,11 @@
       <c r="G19" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H19" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>75</v>
       </c>
@@ -1930,8 +2101,11 @@
       <c r="G20" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H20" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>79</v>
       </c>
@@ -1953,8 +2127,11 @@
       <c r="G21" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H21" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>83</v>
       </c>
@@ -1976,8 +2153,11 @@
       <c r="G22" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H22" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>87</v>
       </c>
@@ -1999,8 +2179,11 @@
       <c r="G23" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H23" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>91</v>
       </c>
@@ -2022,8 +2205,11 @@
       <c r="G24" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H24" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>95</v>
       </c>
@@ -2045,8 +2231,11 @@
       <c r="G25" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H25" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>99</v>
       </c>
@@ -2068,8 +2257,11 @@
       <c r="G26" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H26" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>103</v>
       </c>
@@ -2091,8 +2283,11 @@
       <c r="G27" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H27" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>107</v>
       </c>
@@ -2114,8 +2309,11 @@
       <c r="G28" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H28" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>111</v>
       </c>
@@ -2137,8 +2335,11 @@
       <c r="G29" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H29" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>115</v>
       </c>
@@ -2160,8 +2361,11 @@
       <c r="G30" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H30" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>119</v>
       </c>
@@ -2183,8 +2387,11 @@
       <c r="G31" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H31" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>123</v>
       </c>
@@ -2206,8 +2413,11 @@
       <c r="G32" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H32" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>127</v>
       </c>
@@ -2229,8 +2439,11 @@
       <c r="G33" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H33" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>131</v>
       </c>
@@ -2252,8 +2465,11 @@
       <c r="G34" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H34" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>135</v>
       </c>
@@ -2275,8 +2491,11 @@
       <c r="G35" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H35" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>139</v>
       </c>
@@ -2298,8 +2517,11 @@
       <c r="G36" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H36" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>143</v>
       </c>
@@ -2320,6 +2542,9 @@
       </c>
       <c r="G37" t="s">
         <v>187</v>
+      </c>
+      <c r="H37" t="s">
+        <v>224</v>
       </c>
     </row>
   </sheetData>

</xml_diff>